<commit_message>
Módulos do curso em construção (atualização parcial)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E8e9vSbzJACmFN9asMpEEv
</commit_message>
<xml_diff>
--- a/curso-python/10-dados-com-pandas/dados/planilha_linhas.xlsx
+++ b/curso-python/10-dados-com-pandas/dados/planilha_linhas.xlsx
@@ -502,25 +502,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>004512</t>
+          <t>024412</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>004512-01</t>
+          <t>024412-01</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
         <v>46206</v>
       </c>
       <c r="D3" t="n">
-        <v>47.7</v>
+        <v>38.1</v>
       </c>
       <c r="E3" t="n">
-        <v>44.8</v>
+        <v>36.1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="G3" t="n">
         <v>1558.5</v>
@@ -529,25 +529,25 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>004512</t>
+          <t>024412</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>004512-02</t>
+          <t>024412-02</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
         <v>46208</v>
       </c>
       <c r="D4" t="n">
-        <v>45.6</v>
+        <v>36.4</v>
       </c>
       <c r="E4" t="n">
-        <v>41.7</v>
+        <v>33.4</v>
       </c>
       <c r="F4" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="G4" t="n">
         <v>1256.6</v>
@@ -556,25 +556,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>004512</t>
+          <t>024412</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>004512-03</t>
+          <t>024412-03</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
         <v>46206</v>
       </c>
       <c r="D5" t="n">
-        <v>49.5</v>
+        <v>39.6</v>
       </c>
       <c r="E5" t="n">
-        <v>44.9</v>
+        <v>36</v>
       </c>
       <c r="F5" t="n">
-        <v>0.24</v>
+        <v>0.27</v>
       </c>
       <c r="G5" t="n">
         <v>782.2</v>
@@ -583,25 +583,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>004530</t>
+          <t>024430</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>004530-01</t>
+          <t>024430-01</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
         <v>46219</v>
       </c>
       <c r="D6" t="n">
-        <v>65.40000000000001</v>
+        <v>46.7</v>
       </c>
       <c r="E6" t="n">
-        <v>60.1</v>
+        <v>43.2</v>
       </c>
       <c r="F6" t="n">
-        <v>0.23</v>
+        <v>0.26</v>
       </c>
       <c r="G6" t="n">
         <v>1199.4</v>
@@ -610,79 +610,84 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>004530</t>
+          <t>024430</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>004530-02</t>
+          <t>024430-02</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="D7" t="n">
-        <v>66.7</v>
+        <v>47.7</v>
       </c>
       <c r="E7" t="n">
-        <v>61.5</v>
+        <v>44.3</v>
       </c>
       <c r="F7" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="G7" t="n">
-        <v>1366.6</v>
+        <v>1389.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>004530</t>
+          <t>024430</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>004530-03</t>
+          <t>024430-03</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
         <v>46220</v>
       </c>
       <c r="D8" t="n">
-        <v>68.2</v>
+        <v>48.4</v>
       </c>
       <c r="E8" t="n">
-        <v>61.8</v>
+        <v>44.3</v>
       </c>
       <c r="F8" t="n">
-        <v>0.27</v>
+        <v>0.38</v>
       </c>
       <c r="G8" t="n">
         <v>1362.7</v>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>COF: liberado</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>004530</t>
+          <t>024430</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>004530-04</t>
+          <t>024430-04</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
         <v>46221</v>
       </c>
       <c r="D9" t="n">
-        <v>69.7</v>
+        <v>48.4</v>
       </c>
       <c r="E9" t="n">
-        <v>63.9</v>
+        <v>44.6</v>
       </c>
       <c r="F9" t="n">
-        <v>0.3</v>
+        <v>0.34</v>
       </c>
       <c r="G9" t="n">
         <v>1387.5</v>
@@ -691,25 +696,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>004530</t>
+          <t>024430</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>004530-05</t>
+          <t>024430-05</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
         <v>46219</v>
       </c>
       <c r="D10" t="n">
-        <v>71.09999999999999</v>
+        <v>50.8</v>
       </c>
       <c r="E10" t="n">
-        <v>65</v>
+        <v>46.7</v>
       </c>
       <c r="F10" t="n">
-        <v>0.26</v>
+        <v>0.29</v>
       </c>
       <c r="G10" t="n">
         <v>808.8</v>
@@ -718,25 +723,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>004540</t>
+          <t>024440</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>004540-01</t>
+          <t>024440-01</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
         <v>46232</v>
       </c>
       <c r="D11" t="n">
-        <v>53</v>
+        <v>42.4</v>
       </c>
       <c r="E11" t="n">
-        <v>48.5</v>
+        <v>39</v>
       </c>
       <c r="F11" t="n">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
       <c r="G11" t="n">
         <v>1430.4</v>
@@ -745,25 +750,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>004540</t>
+          <t>024440</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>004540-02</t>
+          <t>024440-02</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
         <v>46232</v>
       </c>
       <c r="D12" t="n">
-        <v>48.8</v>
+        <v>39</v>
       </c>
       <c r="E12" t="n">
-        <v>44.5</v>
+        <v>35.7</v>
       </c>
       <c r="F12" t="n">
-        <v>0.26</v>
+        <v>0.29</v>
       </c>
       <c r="G12" t="n">
         <v>860.2</v>
@@ -772,25 +777,25 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>004540</t>
+          <t>024440</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>004540-03</t>
+          <t>024440-03</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
         <v>46232</v>
       </c>
       <c r="D13" t="n">
-        <v>47.3</v>
+        <v>37.8</v>
       </c>
       <c r="E13" t="n">
-        <v>43.7</v>
+        <v>35.1</v>
       </c>
       <c r="F13" t="n">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="G13" t="n">
         <v>995.6</v>
@@ -799,25 +804,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>004540</t>
+          <t>024440</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>004540-04</t>
+          <t>024440-04</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
         <v>46233</v>
       </c>
       <c r="D14" t="n">
-        <v>47.4</v>
+        <v>37.9</v>
       </c>
       <c r="E14" t="n">
-        <v>43.1</v>
+        <v>34.6</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="G14" t="n">
         <v>1361.6</v>
@@ -826,25 +831,25 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>004562</t>
+          <t>024462</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>004562-01</t>
+          <t>024462-01</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
         <v>46253</v>
       </c>
       <c r="D15" t="n">
-        <v>51.9</v>
+        <v>41.5</v>
       </c>
       <c r="E15" t="n">
-        <v>48.1</v>
+        <v>38.7</v>
       </c>
       <c r="F15" t="n">
-        <v>0.25</v>
+        <v>0.28</v>
       </c>
       <c r="G15" t="n">
         <v>919.5</v>
@@ -853,25 +858,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>004562</t>
+          <t>024462</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>004562-02</t>
+          <t>024462-02</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
         <v>46254</v>
       </c>
       <c r="D16" t="n">
-        <v>47.4</v>
+        <v>37.9</v>
       </c>
       <c r="E16" t="n">
-        <v>43.8</v>
+        <v>35.3</v>
       </c>
       <c r="F16" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="G16" t="n">
         <v>1243.7</v>
@@ -880,25 +885,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>004562</t>
+          <t>024462</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>004562-03</t>
+          <t>024462-03</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
         <v>46254</v>
       </c>
       <c r="D17" t="n">
-        <v>51.5</v>
+        <v>41.2</v>
       </c>
       <c r="E17" t="n">
-        <v>47.1</v>
+        <v>37.8</v>
       </c>
       <c r="F17" t="n">
-        <v>0.25</v>
+        <v>0.28</v>
       </c>
       <c r="G17" t="n">
         <v>1212.9</v>
@@ -907,25 +912,25 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>004570</t>
+          <t>024470</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>004570-01</t>
+          <t>024470-01</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
         <v>46269</v>
       </c>
       <c r="D18" t="n">
-        <v>68.40000000000001</v>
+        <v>48.8</v>
       </c>
       <c r="E18" t="n">
-        <v>62.6</v>
+        <v>44.8</v>
       </c>
       <c r="F18" t="n">
-        <v>0.28</v>
+        <v>0.32</v>
       </c>
       <c r="G18" t="n">
         <v>968.4</v>
@@ -934,25 +939,25 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>004570</t>
+          <t>024470</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>004570-02</t>
+          <t>024470-02</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
         <v>46269</v>
       </c>
       <c r="D19" t="n">
-        <v>68.09999999999999</v>
+        <v>48.7</v>
       </c>
       <c r="E19" t="n">
-        <v>62.4</v>
+        <v>44.9</v>
       </c>
       <c r="F19" t="n">
-        <v>0.24</v>
+        <v>0.27</v>
       </c>
       <c r="G19" t="n">
         <v>1036.4</v>
@@ -961,25 +966,25 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>004570</t>
+          <t>024470</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>004570-03</t>
+          <t>024470-03</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
         <v>46267</v>
       </c>
       <c r="D20" t="n">
-        <v>64.90000000000001</v>
+        <v>46.4</v>
       </c>
       <c r="E20" t="n">
-        <v>59.7</v>
+        <v>42.9</v>
       </c>
       <c r="F20" t="n">
-        <v>0.28</v>
+        <v>0.32</v>
       </c>
       <c r="G20" t="n">
         <v>1459.9</v>
@@ -988,12 +993,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>004583</t>
+          <t>024483</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>004583-01</t>
+          <t>024483-01</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -1006,7 +1011,7 @@
         <v>86.5</v>
       </c>
       <c r="F21" t="n">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
       <c r="G21" t="n">
         <v>1118.5</v>
@@ -1015,12 +1020,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>004583</t>
+          <t>024483</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>004583-02</t>
+          <t>024483-02</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
@@ -1033,7 +1038,7 @@
         <v>86</v>
       </c>
       <c r="F22" t="n">
-        <v>0.24</v>
+        <v>0.27</v>
       </c>
       <c r="G22" t="n">
         <v>1024.8</v>
@@ -1042,12 +1047,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>004583</t>
+          <t>024483</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>004583-03</t>
+          <t>024483-03</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
@@ -1060,7 +1065,7 @@
         <v>78.5</v>
       </c>
       <c r="F23" t="n">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="G23" t="n">
         <v>1038.3</v>
@@ -1069,12 +1074,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>004583</t>
+          <t>024483</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>004583-04</t>
+          <t>024483-04</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -1087,7 +1092,7 @@
         <v>78.7</v>
       </c>
       <c r="F24" t="n">
-        <v>0.33</v>
+        <v>0.37</v>
       </c>
       <c r="G24" t="n">
         <v>1407.9</v>
@@ -1101,12 +1106,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>004583</t>
+          <t>024483</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>004583-05</t>
+          <t>024483-05</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
@@ -1119,7 +1124,7 @@
         <v>84.40000000000001</v>
       </c>
       <c r="F25" t="n">
-        <v>0.27</v>
+        <v>0.31</v>
       </c>
       <c r="G25" t="n">
         <v>812.5</v>
@@ -1128,25 +1133,25 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>004599</t>
+          <t>024499</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>004599-01</t>
+          <t>024499-01</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
         <v>46291</v>
       </c>
       <c r="D26" t="n">
-        <v>52.8</v>
+        <v>42.2</v>
       </c>
       <c r="E26" t="n">
-        <v>48.8</v>
+        <v>39.2</v>
       </c>
       <c r="F26" t="n">
-        <v>0.25</v>
+        <v>0.28</v>
       </c>
       <c r="G26" t="n">
         <v>1345.7</v>
@@ -1155,25 +1160,25 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>004599</t>
+          <t>024499</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>004599-02</t>
+          <t>024499-02</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
         <v>46293</v>
       </c>
       <c r="D27" t="n">
-        <v>52.6</v>
+        <v>42.1</v>
       </c>
       <c r="E27" t="n">
-        <v>48.3</v>
+        <v>38.8</v>
       </c>
       <c r="F27" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="G27" t="n">
         <v>1056.2</v>
@@ -1182,25 +1187,25 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>004599</t>
+          <t>024499</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>004599-03</t>
+          <t>024499-03</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
         <v>46291</v>
       </c>
       <c r="D28" t="n">
-        <v>53.2</v>
+        <v>42.5</v>
       </c>
       <c r="E28" t="n">
-        <v>48.9</v>
+        <v>39.3</v>
       </c>
       <c r="F28" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="G28" t="n">
         <v>1189.4</v>
@@ -1209,25 +1214,25 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>004599</t>
+          <t>024499</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>004599-04</t>
+          <t>024499-04</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
         <v>46292</v>
       </c>
       <c r="D29" t="n">
-        <v>53.3</v>
+        <v>42.7</v>
       </c>
       <c r="E29" t="n">
-        <v>48.9</v>
+        <v>39.4</v>
       </c>
       <c r="F29" t="n">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="G29" t="n">
         <v>1395.3</v>
@@ -1236,25 +1241,25 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>004599</t>
+          <t>024499</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>004599-05</t>
+          <t>024499-05</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
         <v>46293</v>
       </c>
       <c r="D30" t="n">
-        <v>46.1</v>
+        <v>36.9</v>
       </c>
       <c r="E30" t="n">
-        <v>42</v>
+        <v>33.7</v>
       </c>
       <c r="F30" t="n">
-        <v>0.29</v>
+        <v>0.32</v>
       </c>
       <c r="G30" t="n">
         <v>1501.3</v>
@@ -1336,25 +1341,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>004513</t>
+          <t>024413</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>004513-01</t>
+          <t>024413-01</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
         <v>46208</v>
       </c>
       <c r="D3" t="n">
-        <v>18.8</v>
+        <v>32.9</v>
       </c>
       <c r="E3" t="n">
-        <v>17.6</v>
+        <v>31</v>
       </c>
       <c r="F3" t="n">
-        <v>0.33</v>
+        <v>0.37</v>
       </c>
       <c r="G3" t="n">
         <v>790</v>
@@ -1363,25 +1368,25 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>004513</t>
+          <t>024413</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>004513-02</t>
+          <t>024413-02</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
         <v>46208</v>
       </c>
       <c r="D4" t="n">
-        <v>20.8</v>
+        <v>36.4</v>
       </c>
       <c r="E4" t="n">
-        <v>18.5</v>
+        <v>33.4</v>
       </c>
       <c r="F4" t="n">
-        <v>0.28</v>
+        <v>0.3</v>
       </c>
       <c r="G4" t="n">
         <v>1632.5</v>
@@ -1390,25 +1395,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>004513</t>
+          <t>024413</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>004513-03</t>
+          <t>024413-03</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
         <v>46209</v>
       </c>
       <c r="D5" t="n">
-        <v>20.8</v>
+        <v>36.5</v>
       </c>
       <c r="E5" t="n">
-        <v>19.5</v>
+        <v>34.4</v>
       </c>
       <c r="F5" t="n">
-        <v>0.26</v>
+        <v>0.29</v>
       </c>
       <c r="G5" t="n">
         <v>1226.8</v>
@@ -1417,25 +1422,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>004533</t>
+          <t>024433</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>004533-01</t>
+          <t>024433-01</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
         <v>46227</v>
       </c>
       <c r="D6" t="n">
-        <v>21.6</v>
+        <v>37.8</v>
       </c>
       <c r="E6" t="n">
-        <v>20.3</v>
+        <v>35.7</v>
       </c>
       <c r="F6" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="G6" t="n">
         <v>1586.5</v>
@@ -1444,25 +1449,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>004533</t>
+          <t>024433</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>004533-02</t>
+          <t>024433-02</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
         <v>46226</v>
       </c>
       <c r="D7" t="n">
-        <v>19.6</v>
+        <v>34.3</v>
       </c>
       <c r="E7" t="n">
-        <v>17.9</v>
+        <v>32</v>
       </c>
       <c r="F7" t="n">
-        <v>0.28</v>
+        <v>0.3</v>
       </c>
       <c r="G7" t="n">
         <v>1482.9</v>
@@ -1471,25 +1476,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>004533</t>
+          <t>024433</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>004533-03</t>
+          <t>024433-03</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
         <v>46226</v>
       </c>
       <c r="D8" t="n">
-        <v>19.1</v>
+        <v>33.3</v>
       </c>
       <c r="E8" t="n">
-        <v>16.5</v>
+        <v>30</v>
       </c>
       <c r="F8" t="n">
-        <v>0.26</v>
+        <v>0.29</v>
       </c>
       <c r="G8" t="n">
         <v>1055.5</v>
@@ -1498,25 +1503,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>004533</t>
+          <t>024433</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>004533-04</t>
+          <t>024433-04</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
         <v>46227</v>
       </c>
       <c r="D9" t="n">
-        <v>20.4</v>
+        <v>35.6</v>
       </c>
       <c r="E9" t="n">
-        <v>18.4</v>
+        <v>32.9</v>
       </c>
       <c r="F9" t="n">
-        <v>0.27</v>
+        <v>0.29</v>
       </c>
       <c r="G9" t="n">
         <v>1005.2</v>
@@ -1525,25 +1530,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>004533</t>
+          <t>024433</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>004533-05</t>
+          <t>024433-05</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
         <v>46226</v>
       </c>
       <c r="D10" t="n">
-        <v>18.5</v>
+        <v>32.4</v>
       </c>
       <c r="E10" t="n">
-        <v>17</v>
+        <v>30.2</v>
       </c>
       <c r="F10" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="G10" t="n">
         <v>1512.9</v>
@@ -1552,25 +1557,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>004558</t>
+          <t>024458</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>004558-01</t>
+          <t>024458-01</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
         <v>46248</v>
       </c>
       <c r="D11" t="n">
-        <v>19.9</v>
+        <v>34.8</v>
       </c>
       <c r="E11" t="n">
-        <v>17.9</v>
+        <v>32.1</v>
       </c>
       <c r="F11" t="n">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="G11" t="n">
         <v>809.7</v>
@@ -1579,25 +1584,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>004558</t>
+          <t>024458</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>004558-02</t>
+          <t>024458-02</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
         <v>46247</v>
       </c>
       <c r="D12" t="n">
-        <v>19.7</v>
+        <v>34.4</v>
       </c>
       <c r="E12" t="n">
-        <v>17.6</v>
+        <v>31.6</v>
       </c>
       <c r="F12" t="n">
-        <v>0.24</v>
+        <v>0.44</v>
       </c>
       <c r="G12" t="n">
         <v>1173.1</v>
@@ -1606,25 +1611,25 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>004558</t>
+          <t>024458</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>004558-03</t>
+          <t>024458-03</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
         <v>46249</v>
       </c>
       <c r="D13" t="n">
-        <v>18.3</v>
+        <v>32.1</v>
       </c>
       <c r="E13" t="n">
-        <v>16.6</v>
+        <v>29.7</v>
       </c>
       <c r="F13" t="n">
-        <v>0.27</v>
+        <v>0.29</v>
       </c>
       <c r="G13" t="n">
         <v>1370.4</v>
@@ -1633,25 +1638,25 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>004579</t>
+          <t>024479</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>004579-01</t>
+          <t>024479-01</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
         <v>46275</v>
       </c>
       <c r="D14" t="n">
-        <v>20.6</v>
+        <v>36.1</v>
       </c>
       <c r="E14" t="n">
-        <v>18.6</v>
+        <v>33.4</v>
       </c>
       <c r="F14" t="n">
-        <v>0.29</v>
+        <v>0.32</v>
       </c>
       <c r="G14" t="n">
         <v>984.6</v>
@@ -1660,25 +1665,25 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>004579</t>
+          <t>024479</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>004579-02</t>
+          <t>024479-02</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
         <v>46276</v>
       </c>
       <c r="D15" t="n">
-        <v>19.9</v>
+        <v>34.7</v>
       </c>
       <c r="E15" t="n">
-        <v>18.2</v>
+        <v>32.3</v>
       </c>
       <c r="F15" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="G15" t="n">
         <v>1054</v>
@@ -1687,25 +1692,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>004579</t>
+          <t>024479</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>004579-03</t>
+          <t>024479-03</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
         <v>46277</v>
       </c>
       <c r="D16" t="n">
-        <v>19</v>
+        <v>33.2</v>
       </c>
       <c r="E16" t="n">
-        <v>16.7</v>
+        <v>30.2</v>
       </c>
       <c r="F16" t="n">
-        <v>0.3</v>
+        <v>0.34</v>
       </c>
       <c r="G16" t="n">
         <v>1315.2</v>
@@ -1714,25 +1719,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>004579</t>
+          <t>024479</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>004579-04</t>
+          <t>024479-04</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
         <v>46277</v>
       </c>
       <c r="D17" t="n">
-        <v>20.7</v>
+        <v>36.2</v>
       </c>
       <c r="E17" t="n">
-        <v>18.6</v>
+        <v>33.4</v>
       </c>
       <c r="F17" t="n">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="G17" t="n">
         <v>1544.2</v>
@@ -1814,25 +1819,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>004520</t>
+          <t>024420</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>004520-01</t>
+          <t>024420-01</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
         <v>46212</v>
       </c>
       <c r="D3" t="n">
-        <v>12</v>
+        <v>69.8</v>
       </c>
       <c r="E3" t="n">
-        <v>16.5</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>0.31</v>
+        <v>0.19</v>
       </c>
       <c r="G3" t="n">
         <v>1542.5</v>
@@ -1841,25 +1846,25 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>004520</t>
+          <t>024420</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>004520-02</t>
+          <t>024420-02</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
         <v>46212</v>
       </c>
       <c r="D4" t="n">
-        <v>11.9</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>16.4</v>
+        <v>64.3</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3</v>
+        <v>0.17</v>
       </c>
       <c r="G4" t="n">
         <v>1517.6</v>
@@ -1868,52 +1873,57 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>004520</t>
+          <t>024420</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>004520-03</t>
+          <t>024420-03</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
         <v>46214</v>
       </c>
       <c r="D5" t="n">
-        <v>11.6</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>16.5</v>
+        <v>63.1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4</v>
+        <v>0.34</v>
       </c>
       <c r="G5" t="n">
         <v>1213.7</v>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>COF: liberado</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>004551</t>
+          <t>024451</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>004551-01</t>
+          <t>024451-01</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
         <v>46242</v>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>69.7</v>
       </c>
       <c r="E6" t="n">
-        <v>16.8</v>
+        <v>64.8</v>
       </c>
       <c r="F6" t="n">
-        <v>0.33</v>
+        <v>0.21</v>
       </c>
       <c r="G6" t="n">
         <v>1342.3</v>
@@ -1922,25 +1932,25 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>004551</t>
+          <t>024451</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>004551-02</t>
+          <t>024451-02</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
         <v>46243</v>
       </c>
       <c r="D7" t="n">
-        <v>13.2</v>
+        <v>77</v>
       </c>
       <c r="E7" t="n">
-        <v>18</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>0.38</v>
+        <v>0.26</v>
       </c>
       <c r="G7" t="n">
         <v>1044.2</v>
@@ -1949,25 +1959,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>004551</t>
+          <t>024451</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>004551-03</t>
+          <t>024451-03</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
         <v>46242</v>
       </c>
       <c r="D8" t="n">
-        <v>12.1</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>16.7</v>
+        <v>65.5</v>
       </c>
       <c r="F8" t="n">
-        <v>0.36</v>
+        <v>0.24</v>
       </c>
       <c r="G8" t="n">
         <v>1277.3</v>
@@ -1976,25 +1986,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>004551</t>
+          <t>024451</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>004551-04</t>
+          <t>024451-04</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
         <v>46242</v>
       </c>
       <c r="D9" t="n">
-        <v>12.1</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="E9" t="n">
-        <v>16.6</v>
+        <v>65.3</v>
       </c>
       <c r="F9" t="n">
-        <v>0.3</v>
+        <v>0.18</v>
       </c>
       <c r="G9" t="n">
         <v>1179.2</v>
@@ -2003,25 +2013,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>004574</t>
+          <t>024474</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>004574-01</t>
+          <t>024474-01</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
         <v>46271</v>
       </c>
       <c r="D10" t="n">
-        <v>12.3</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>17</v>
+        <v>66.7</v>
       </c>
       <c r="F10" t="n">
-        <v>0.32</v>
+        <v>0.19</v>
       </c>
       <c r="G10" t="n">
         <v>1478</v>
@@ -2030,25 +2040,25 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>004574</t>
+          <t>024474</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>004574-02</t>
+          <t>024474-02</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
         <v>46270</v>
       </c>
       <c r="D11" t="n">
-        <v>11.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>15.5</v>
+        <v>60.3</v>
       </c>
       <c r="F11" t="n">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="G11" t="n">
         <v>1020.8</v>
@@ -2057,25 +2067,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>004574</t>
+          <t>024474</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>004574-03</t>
+          <t>024474-03</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
         <v>46269</v>
       </c>
       <c r="D12" t="n">
-        <v>12.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>16.7</v>
+        <v>66</v>
       </c>
       <c r="F12" t="n">
-        <v>0.33</v>
+        <v>0.21</v>
       </c>
       <c r="G12" t="n">
         <v>792.1</v>
@@ -2157,12 +2167,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>004521</t>
+          <t>024421</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>004521-01</t>
+          <t>024421-01</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
@@ -2175,7 +2185,7 @@
         <v>65.3</v>
       </c>
       <c r="F3" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="G3" t="n">
         <v>1541.6</v>
@@ -2184,12 +2194,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>004521</t>
+          <t>024421</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>004521-02</t>
+          <t>024421-02</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
@@ -2202,7 +2212,7 @@
         <v>60.3</v>
       </c>
       <c r="F4" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="G4" t="n">
         <v>1226.3</v>
@@ -2211,12 +2221,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>004521</t>
+          <t>024421</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>004521-03</t>
+          <t>024421-03</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -2229,7 +2239,7 @@
         <v>59.8</v>
       </c>
       <c r="F5" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="G5" t="n">
         <v>1491.8</v>
@@ -2238,12 +2248,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>004547</t>
+          <t>024447</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>004547-01</t>
+          <t>024447-01</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -2256,7 +2266,7 @@
         <v>62.5</v>
       </c>
       <c r="F6" t="n">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="G6" t="n">
         <v>1380.1</v>
@@ -2265,12 +2275,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>004547</t>
+          <t>024447</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>004547-02</t>
+          <t>024447-02</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
@@ -2283,7 +2293,7 @@
         <v>60</v>
       </c>
       <c r="F7" t="n">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="G7" t="n">
         <v>1291.5</v>
@@ -2292,12 +2302,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>004547</t>
+          <t>024447</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>004547-03</t>
+          <t>024447-03</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
@@ -2310,7 +2320,7 @@
         <v>68.09999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="G8" t="n">
         <v>919.3</v>
@@ -2319,12 +2329,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>004547</t>
+          <t>024447</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>004547-04</t>
+          <t>024447-04</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
@@ -2337,7 +2347,7 @@
         <v>63.2</v>
       </c>
       <c r="F9" t="n">
-        <v>0.24</v>
+        <v>0.27</v>
       </c>
       <c r="G9" t="n">
         <v>1046.2</v>
@@ -2346,12 +2356,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>004547</t>
+          <t>024447</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>004547-05</t>
+          <t>024447-05</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
@@ -2364,7 +2374,7 @@
         <v>58.7</v>
       </c>
       <c r="F10" t="n">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="G10" t="n">
         <v>1614.2</v>
@@ -2373,12 +2383,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>004566</t>
+          <t>024466</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>004566-01</t>
+          <t>024466-01</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -2391,7 +2401,7 @@
         <v>64.3</v>
       </c>
       <c r="F11" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="G11" t="n">
         <v>1199.4</v>
@@ -2400,12 +2410,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>004566</t>
+          <t>024466</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>004566-02</t>
+          <t>024466-02</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
@@ -2418,7 +2428,7 @@
         <v>66.8</v>
       </c>
       <c r="F12" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="G12" t="n">
         <v>981.3</v>
@@ -2427,12 +2437,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>004566</t>
+          <t>024466</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>004566-03</t>
+          <t>024466-03</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
@@ -2445,7 +2455,7 @@
         <v>58.5</v>
       </c>
       <c r="F13" t="n">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="G13" t="n">
         <v>1067.5</v>
@@ -2454,12 +2464,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>004566</t>
+          <t>024466</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>004566-04</t>
+          <t>024466-04</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
@@ -2472,7 +2482,7 @@
         <v>57.3</v>
       </c>
       <c r="F14" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="G14" t="n">
         <v>1086.2</v>
@@ -2481,12 +2491,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>004588</t>
+          <t>024488</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>004588-01</t>
+          <t>024488-01</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -2499,7 +2509,7 @@
         <v>60.6</v>
       </c>
       <c r="F15" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="G15" t="n">
         <v>889.9</v>
@@ -2508,12 +2518,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>004588</t>
+          <t>024488</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>004588-02</t>
+          <t>024488-02</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -2526,7 +2536,7 @@
         <v>61.8</v>
       </c>
       <c r="F16" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="G16" t="n">
         <v>1356.5</v>
@@ -2535,12 +2545,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>004588</t>
+          <t>024488</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>004588-03</t>
+          <t>024488-03</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
@@ -2553,7 +2563,7 @@
         <v>62.8</v>
       </c>
       <c r="F17" t="n">
-        <v>0.24</v>
+        <v>0.28</v>
       </c>
       <c r="G17" t="n">
         <v>1374.9</v>
@@ -2562,12 +2572,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>004588</t>
+          <t>024488</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>004588-04</t>
+          <t>024488-04</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -2580,7 +2590,7 @@
         <v>63.3</v>
       </c>
       <c r="F18" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="G18" t="n">
         <v>978.6</v>
@@ -2589,12 +2599,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>004588</t>
+          <t>024488</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>004588-05</t>
+          <t>024488-05</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -2607,7 +2617,7 @@
         <v>66.3</v>
       </c>
       <c r="F19" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="G19" t="n">
         <v>1601.5</v>

</xml_diff>